<commit_message>
Serie C: calendario FIR rev. 28/09 — Bergamo 1950 al campo Utili (05/12, 17/04 h.19), orari G3/G7
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Risultati_Serie_B-C_2026-27.xlsx
+++ b/Risultati_Serie_B-C_2026-27.xlsx
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -101,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -110,7 +109,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -123,6 +122,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -573,7 +575,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="9" t="n">
         <v>46313</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -618,7 +620,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="9" t="n">
         <v>46313</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -659,7 +661,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="9" t="n">
         <v>46313</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -700,7 +702,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="9" t="n">
         <v>46313</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -741,7 +743,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="9" t="n">
         <v>46313</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -782,7 +784,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="9" t="n">
         <v>46320</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -823,7 +825,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="9" t="n">
         <v>46320</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -864,7 +866,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="9" t="n">
         <v>46320</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -905,7 +907,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="9" t="n">
         <v>46320</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -946,7 +948,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="9" t="n">
         <v>46320</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -987,7 +989,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="9" t="n">
         <v>46334</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1028,7 +1030,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="9" t="n">
         <v>46334</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1069,7 +1071,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="9" t="n">
         <v>46334</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1110,7 +1112,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="9" t="n">
         <v>46334</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1151,7 +1153,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="9" t="n">
         <v>46334</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1192,7 +1194,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="9" t="n">
         <v>46341</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1233,7 +1235,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C20" s="9" t="n">
         <v>46341</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1274,7 +1276,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="9" t="n">
         <v>46341</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1315,7 +1317,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n">
+      <c r="C22" s="9" t="n">
         <v>46341</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1356,7 +1358,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C23" s="9" t="n">
         <v>46341</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1397,7 +1399,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="C24" s="9" t="n">
         <v>46355</v>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1438,7 +1440,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C25" s="9" t="n">
         <v>46355</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1479,7 +1481,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C26" s="4" t="n">
+      <c r="C26" s="9" t="n">
         <v>46355</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1520,7 +1522,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="C27" s="9" t="n">
         <v>46355</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1561,7 +1563,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C28" s="4" t="n">
+      <c r="C28" s="9" t="n">
         <v>46355</v>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1602,7 +1604,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C29" s="4" t="n">
+      <c r="C29" s="9" t="n">
         <v>46362</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1643,7 +1645,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C30" s="4" t="n">
+      <c r="C30" s="9" t="n">
         <v>46362</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1684,7 +1686,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n">
+      <c r="C31" s="9" t="n">
         <v>46362</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1725,7 +1727,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C32" s="4" t="n">
+      <c r="C32" s="9" t="n">
         <v>46362</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1766,7 +1768,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C33" s="4" t="n">
+      <c r="C33" s="9" t="n">
         <v>46362</v>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1807,7 +1809,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C34" s="4" t="n">
+      <c r="C34" s="9" t="n">
         <v>46369</v>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -1848,7 +1850,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="C35" s="9" t="n">
         <v>46369</v>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1889,7 +1891,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C36" s="4" t="n">
+      <c r="C36" s="9" t="n">
         <v>46369</v>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1930,7 +1932,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C37" s="4" t="n">
+      <c r="C37" s="9" t="n">
         <v>46369</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1971,7 +1973,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C38" s="4" t="n">
+      <c r="C38" s="9" t="n">
         <v>46369</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -2012,7 +2014,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C39" s="4" t="n">
+      <c r="C39" s="9" t="n">
         <v>46404</v>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -2053,7 +2055,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C40" s="4" t="n">
+      <c r="C40" s="9" t="n">
         <v>46404</v>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -2094,7 +2096,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C41" s="4" t="n">
+      <c r="C41" s="9" t="n">
         <v>46404</v>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -2135,7 +2137,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C42" s="4" t="n">
+      <c r="C42" s="9" t="n">
         <v>46404</v>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -2176,7 +2178,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C43" s="4" t="n">
+      <c r="C43" s="9" t="n">
         <v>46404</v>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -2217,7 +2219,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C44" s="4" t="n">
+      <c r="C44" s="9" t="n">
         <v>46411</v>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -2258,7 +2260,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C45" s="4" t="n">
+      <c r="C45" s="9" t="n">
         <v>46411</v>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -2299,7 +2301,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C46" s="4" t="n">
+      <c r="C46" s="9" t="n">
         <v>46411</v>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -2340,7 +2342,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C47" s="4" t="n">
+      <c r="C47" s="9" t="n">
         <v>46411</v>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -2381,7 +2383,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C48" s="4" t="n">
+      <c r="C48" s="9" t="n">
         <v>46411</v>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -2422,7 +2424,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C49" s="4" t="n">
+      <c r="C49" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -2463,7 +2465,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C50" s="4" t="n">
+      <c r="C50" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -2504,7 +2506,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C51" s="4" t="n">
+      <c r="C51" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -2545,7 +2547,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C52" s="4" t="n">
+      <c r="C52" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -2586,7 +2588,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C53" s="4" t="n">
+      <c r="C53" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -2627,7 +2629,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C54" s="4" t="n">
+      <c r="C54" s="9" t="n">
         <v>46439</v>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -2668,7 +2670,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C55" s="4" t="n">
+      <c r="C55" s="9" t="n">
         <v>46439</v>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -2709,7 +2711,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C56" s="4" t="n">
+      <c r="C56" s="9" t="n">
         <v>46439</v>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -2750,7 +2752,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C57" s="4" t="n">
+      <c r="C57" s="9" t="n">
         <v>46439</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -2791,7 +2793,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C58" s="4" t="n">
+      <c r="C58" s="9" t="n">
         <v>46439</v>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -2832,7 +2834,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C59" s="4" t="n">
+      <c r="C59" s="9" t="n">
         <v>46446</v>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -2873,7 +2875,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C60" s="4" t="n">
+      <c r="C60" s="9" t="n">
         <v>46446</v>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2914,7 +2916,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C61" s="4" t="n">
+      <c r="C61" s="9" t="n">
         <v>46446</v>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2955,7 +2957,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C62" s="4" t="n">
+      <c r="C62" s="9" t="n">
         <v>46446</v>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -2996,7 +2998,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C63" s="4" t="n">
+      <c r="C63" s="9" t="n">
         <v>46446</v>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -3037,7 +3039,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C64" s="4" t="n">
+      <c r="C64" s="9" t="n">
         <v>46467</v>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -3078,7 +3080,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C65" s="4" t="n">
+      <c r="C65" s="9" t="n">
         <v>46467</v>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -3119,7 +3121,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C66" s="4" t="n">
+      <c r="C66" s="9" t="n">
         <v>46467</v>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -3160,7 +3162,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C67" s="4" t="n">
+      <c r="C67" s="9" t="n">
         <v>46467</v>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -3201,7 +3203,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C68" s="4" t="n">
+      <c r="C68" s="9" t="n">
         <v>46467</v>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -3242,7 +3244,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C69" s="4" t="n">
+      <c r="C69" s="9" t="n">
         <v>46481</v>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -3283,7 +3285,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C70" s="4" t="n">
+      <c r="C70" s="9" t="n">
         <v>46481</v>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -3324,7 +3326,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C71" s="4" t="n">
+      <c r="C71" s="9" t="n">
         <v>46481</v>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -3365,7 +3367,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C72" s="4" t="n">
+      <c r="C72" s="9" t="n">
         <v>46481</v>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -3406,7 +3408,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C73" s="4" t="n">
+      <c r="C73" s="9" t="n">
         <v>46481</v>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -3447,7 +3449,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C74" s="4" t="n">
+      <c r="C74" s="9" t="n">
         <v>46488</v>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -3488,7 +3490,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C75" s="4" t="n">
+      <c r="C75" s="9" t="n">
         <v>46488</v>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -3529,7 +3531,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C76" s="4" t="n">
+      <c r="C76" s="9" t="n">
         <v>46488</v>
       </c>
       <c r="D76" s="3" t="inlineStr">
@@ -3570,7 +3572,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C77" s="4" t="n">
+      <c r="C77" s="9" t="n">
         <v>46488</v>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -3611,7 +3613,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C78" s="4" t="n">
+      <c r="C78" s="9" t="n">
         <v>46488</v>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -3652,7 +3654,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C79" s="4" t="n">
+      <c r="C79" s="9" t="n">
         <v>46495</v>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -3693,7 +3695,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C80" s="4" t="n">
+      <c r="C80" s="9" t="n">
         <v>46495</v>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -3734,7 +3736,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C81" s="4" t="n">
+      <c r="C81" s="9" t="n">
         <v>46495</v>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -3775,7 +3777,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C82" s="4" t="n">
+      <c r="C82" s="9" t="n">
         <v>46495</v>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -3816,7 +3818,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C83" s="4" t="n">
+      <c r="C83" s="9" t="n">
         <v>46495</v>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -3857,7 +3859,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C84" s="4" t="n">
+      <c r="C84" s="9" t="n">
         <v>46516</v>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -3898,7 +3900,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C85" s="4" t="n">
+      <c r="C85" s="9" t="n">
         <v>46516</v>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -3939,7 +3941,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C86" s="4" t="n">
+      <c r="C86" s="9" t="n">
         <v>46516</v>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -3980,7 +3982,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C87" s="4" t="n">
+      <c r="C87" s="9" t="n">
         <v>46516</v>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -4021,7 +4023,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C88" s="4" t="n">
+      <c r="C88" s="9" t="n">
         <v>46516</v>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -4062,7 +4064,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C89" s="4" t="n">
+      <c r="C89" s="9" t="n">
         <v>46523</v>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -4103,7 +4105,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C90" s="4" t="n">
+      <c r="C90" s="9" t="n">
         <v>46523</v>
       </c>
       <c r="D90" s="3" t="inlineStr">
@@ -4144,7 +4146,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C91" s="4" t="n">
+      <c r="C91" s="9" t="n">
         <v>46523</v>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -4185,7 +4187,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C92" s="4" t="n">
+      <c r="C92" s="9" t="n">
         <v>46523</v>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -4226,7 +4228,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C93" s="4" t="n">
+      <c r="C93" s="9" t="n">
         <v>46523</v>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -4369,7 +4371,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="9" t="n">
         <v>46313</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -4414,7 +4416,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="9" t="n">
         <v>46313</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -4455,7 +4457,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="9" t="n">
         <v>46313</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -4496,7 +4498,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="9" t="n">
         <v>46313</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -4537,7 +4539,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="9" t="n">
         <v>46320</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -4578,7 +4580,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="9" t="n">
         <v>46320</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -4619,7 +4621,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="9" t="n">
         <v>46320</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -4660,7 +4662,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="9" t="n">
         <v>46320</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -4701,12 +4703,12 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="9" t="n">
         <v>46327</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -4742,7 +4744,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="9" t="n">
         <v>46327</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -4783,7 +4785,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="9" t="n">
         <v>46327</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -4824,7 +4826,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="9" t="n">
         <v>46327</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -4865,7 +4867,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="9" t="n">
         <v>46348</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -4906,7 +4908,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="9" t="n">
         <v>46348</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -4947,7 +4949,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="9" t="n">
         <v>46348</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -4988,7 +4990,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="9" t="n">
         <v>46348</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -5029,7 +5031,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C20" s="9" t="n">
         <v>46355</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -5070,7 +5072,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="9" t="n">
         <v>46355</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -5111,7 +5113,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n">
+      <c r="C22" s="9" t="n">
         <v>46355</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -5152,7 +5154,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C23" s="9" t="n">
         <v>46355</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -5193,12 +5195,12 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n">
-        <v>46362</v>
+      <c r="C24" s="9" t="n">
+        <v>46361</v>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -5215,7 +5217,7 @@
       <c r="H24" s="6" t="n"/>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Bergamo</t>
+          <t>Bergamo (campo Utili)</t>
         </is>
       </c>
       <c r="J24" s="7">
@@ -5234,7 +5236,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C25" s="9" t="n">
         <v>46362</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -5275,7 +5277,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C26" s="4" t="n">
+      <c r="C26" s="9" t="n">
         <v>46362</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -5316,7 +5318,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="C27" s="9" t="n">
         <v>46362</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -5357,7 +5359,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C28" s="4" t="n">
+      <c r="C28" s="9" t="n">
         <v>46369</v>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -5398,7 +5400,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C29" s="4" t="n">
+      <c r="C29" s="9" t="n">
         <v>46369</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -5439,12 +5441,12 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C30" s="4" t="n">
+      <c r="C30" s="9" t="n">
         <v>46369</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -5480,7 +5482,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n">
+      <c r="C31" s="9" t="n">
         <v>46369</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -5521,7 +5523,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C32" s="4" t="n">
+      <c r="C32" s="9" t="n">
         <v>46404</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -5562,7 +5564,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C33" s="4" t="n">
+      <c r="C33" s="9" t="n">
         <v>46404</v>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -5603,7 +5605,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C34" s="4" t="n">
+      <c r="C34" s="9" t="n">
         <v>46404</v>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -5644,7 +5646,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="C35" s="9" t="n">
         <v>46404</v>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -5685,7 +5687,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C36" s="4" t="n">
+      <c r="C36" s="9" t="n">
         <v>46411</v>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -5726,7 +5728,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C37" s="4" t="n">
+      <c r="C37" s="9" t="n">
         <v>46411</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -5767,7 +5769,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C38" s="4" t="n">
+      <c r="C38" s="9" t="n">
         <v>46411</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -5808,7 +5810,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C39" s="4" t="n">
+      <c r="C39" s="9" t="n">
         <v>46411</v>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -5849,7 +5851,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C40" s="4" t="n">
+      <c r="C40" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -5890,7 +5892,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C41" s="4" t="n">
+      <c r="C41" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -5931,7 +5933,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C42" s="4" t="n">
+      <c r="C42" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -5972,7 +5974,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C43" s="4" t="n">
+      <c r="C43" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -6013,7 +6015,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C44" s="4" t="n">
+      <c r="C44" s="9" t="n">
         <v>46425</v>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -6054,7 +6056,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C45" s="4" t="n">
+      <c r="C45" s="9" t="n">
         <v>46425</v>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -6095,7 +6097,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C46" s="4" t="n">
+      <c r="C46" s="9" t="n">
         <v>46425</v>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -6136,7 +6138,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C47" s="4" t="n">
+      <c r="C47" s="9" t="n">
         <v>46425</v>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -6177,7 +6179,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C48" s="4" t="n">
+      <c r="C48" s="9" t="n">
         <v>46439</v>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -6218,7 +6220,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C49" s="4" t="n">
+      <c r="C49" s="9" t="n">
         <v>46439</v>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -6259,7 +6261,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C50" s="4" t="n">
+      <c r="C50" s="9" t="n">
         <v>46439</v>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -6300,7 +6302,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C51" s="4" t="n">
+      <c r="C51" s="9" t="n">
         <v>46439</v>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -6341,7 +6343,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C52" s="4" t="n">
+      <c r="C52" s="9" t="n">
         <v>46446</v>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -6382,7 +6384,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C53" s="4" t="n">
+      <c r="C53" s="9" t="n">
         <v>46446</v>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -6423,7 +6425,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C54" s="4" t="n">
+      <c r="C54" s="9" t="n">
         <v>46446</v>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -6464,7 +6466,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C55" s="4" t="n">
+      <c r="C55" s="9" t="n">
         <v>46446</v>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -6505,7 +6507,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C56" s="4" t="n">
+      <c r="C56" s="9" t="n">
         <v>46467</v>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -6546,7 +6548,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C57" s="4" t="n">
+      <c r="C57" s="9" t="n">
         <v>46467</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -6587,7 +6589,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C58" s="4" t="n">
+      <c r="C58" s="9" t="n">
         <v>46467</v>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -6628,7 +6630,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C59" s="4" t="n">
+      <c r="C59" s="9" t="n">
         <v>46467</v>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -6669,7 +6671,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C60" s="4" t="n">
+      <c r="C60" s="9" t="n">
         <v>46481</v>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -6710,7 +6712,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C61" s="4" t="n">
+      <c r="C61" s="9" t="n">
         <v>46481</v>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -6751,7 +6753,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C62" s="4" t="n">
+      <c r="C62" s="9" t="n">
         <v>46481</v>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -6792,7 +6794,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C63" s="4" t="n">
+      <c r="C63" s="9" t="n">
         <v>46481</v>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -6833,7 +6835,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C64" s="4" t="n">
+      <c r="C64" s="9" t="n">
         <v>46488</v>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -6874,7 +6876,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C65" s="4" t="n">
+      <c r="C65" s="9" t="n">
         <v>46488</v>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -6915,7 +6917,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C66" s="4" t="n">
+      <c r="C66" s="9" t="n">
         <v>46488</v>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -6956,7 +6958,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C67" s="4" t="n">
+      <c r="C67" s="9" t="n">
         <v>46488</v>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -6997,12 +6999,12 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C68" s="4" t="n">
-        <v>46495</v>
+      <c r="C68" s="9" t="n">
+        <v>46494</v>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -7019,7 +7021,7 @@
       <c r="H68" s="6" t="n"/>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Bergamo</t>
+          <t>Bergamo (campo Utili)</t>
         </is>
       </c>
       <c r="J68" s="7">
@@ -7038,7 +7040,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C69" s="4" t="n">
+      <c r="C69" s="9" t="n">
         <v>46495</v>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -7079,7 +7081,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C70" s="4" t="n">
+      <c r="C70" s="9" t="n">
         <v>46495</v>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -7120,7 +7122,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C71" s="4" t="n">
+      <c r="C71" s="9" t="n">
         <v>46495</v>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -7161,7 +7163,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C72" s="4" t="n">
+      <c r="C72" s="9" t="n">
         <v>46502</v>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -7202,7 +7204,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C73" s="4" t="n">
+      <c r="C73" s="9" t="n">
         <v>46502</v>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -7243,7 +7245,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C74" s="4" t="n">
+      <c r="C74" s="9" t="n">
         <v>46502</v>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -7284,7 +7286,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C75" s="4" t="n">
+      <c r="C75" s="9" t="n">
         <v>46502</v>
       </c>
       <c r="D75" s="3" t="inlineStr">

</xml_diff>